<commit_message>
Update with simulated data
</commit_message>
<xml_diff>
--- a/Synthetic_images/listnames.xlsx
+++ b/Synthetic_images/listnames.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\valad\Documents\GitHub\4polar_3D_SMOLM_simulation\Synthetic_images\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FB19D726-6F30-4F24-B46E-284648BD4A06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58703E98-F924-4F36-9D51-764116F5CB3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3075" yWindow="2355" windowWidth="12885" windowHeight="10095" xr2:uid="{F7587F97-AFB4-448F-A333-4B06CD421373}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F7587F97-AFB4-448F-A333-4B06CD421373}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
     <t>Filenames</t>
   </si>
   <si>
-    <t>Image_ITtheory_10000_r_1p7_w_17_wGen_51_bg_10_delta_001_rho_030_eta_000_lambda_0.6_f_0_z_0_All_PoissonNoise.mat</t>
+    <t>Image_ITtheory_5000_wGen_17_bg_10_delta_100_rho_030_eta_020_lambda_0p6_All_GaussNoise_bin.mat</t>
   </si>
 </sst>
 </file>

</xml_diff>